<commit_message>
Cleaned up spreadsheet files, with full citations added
</commit_message>
<xml_diff>
--- a/figures/Figure3/data/melt_inclusions/Fuego_Data.xlsx
+++ b/figures/Figure3/data/melt_inclusions/Fuego_Data.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiacovino/PythonGit/EoV_CH2-2/figures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiacovino/PythonGit/EoV_CH2-2/figures/Figure3/data/melt_inclusions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{437EA086-89E4-9748-AA89-098C2BBC8D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA0F6A4-76DF-4A45-85B5-67EC1F8B4E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9880" yWindow="2680" windowWidth="32780" windowHeight="22240" xr2:uid="{73286055-14FF-C145-B2C7-067475171440}"/>
+    <workbookView xWindow="13220" yWindow="34560" windowWidth="32780" windowHeight="21700" xr2:uid="{73286055-14FF-C145-B2C7-067475171440}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Citations" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="65">
   <si>
     <t>Volcano</t>
   </si>
@@ -225,13 +226,99 @@
   </si>
   <si>
     <t>CO2</t>
+  </si>
+  <si>
+    <r>
+      <t>Moore, L.R., E. Gazel, R. Tuohy, A.S. Lloyd, R. Esposito, M. Steele-MacInnis, E.H. Hauri, P.J. Wallace, T. Plank, and R.J. Bodnar, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bubbles matter: An assessment of the contribution of vapor bubbles to melt inclusion volatile budgets.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> American Mineralogist, 2015. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(4): p. 806-823.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Lloyd, A.S., T. Plank, P. Ruprecht, E.H. Hauri, and W. Rose, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Volatile loss from melt inclusions in pyroclasts of differing sizes.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Contributions to Mineralogy and Petrology, 2013. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>165</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(1): p. 129-153.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -258,6 +345,26 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -279,11 +386,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3262,4 +3370,34 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BC1FF33-AC79-EF49-BFD4-202DF60F05C1}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="236.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>